<commit_message>
update/redo testoutput files with slight change in rounding of latlon in urls etc
</commit_message>
<xml_diff>
--- a/inst/testdata/examples_of_output/testoutput_ejam2excel_fips_cities.xlsx
+++ b/inst/testdata/examples_of_output/testoutput_ejam2excel_fips_cities.xlsx
@@ -38,7 +38,7 @@
     <t xml:space="preserve">Locations analyzed</t>
   </si>
   <si>
-    <t xml:space="preserve">Census Units defined by FIPS code</t>
+    <t xml:space="preserve">Selected Locations</t>
   </si>
   <si>
     <t xml:space="preserve">Distance in miles</t>
@@ -50,13 +50,13 @@
     <t xml:space="preserve">Distance type</t>
   </si>
   <si>
-    <t xml:space="preserve">Miles radius of circular buffer (or distance used if buffering around polygons)</t>
+    <t xml:space="preserve">Residents within any of the 2 specified cities. Area in Square Miles: 88.36</t>
   </si>
   <si>
     <t xml:space="preserve">Population at x% of sites</t>
   </si>
   <si>
-    <t xml:space="preserve">0% of places account for 50% of the total population (approx.)</t>
+    <t xml:space="preserve">The most-populated 50% of the 2 places can account for at least 50% of the total population of all sites as a whole.</t>
   </si>
   <si>
     <t xml:space="preserve">Population at N sites</t>
@@ -1502,10 +1502,10 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?fips=2743000&amp;buffer=0&amp;sitenumber=-1&amp;sitetype=fips&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=44.9634699531927,-93.2677936369264", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?fips=2743000&amp;buffer=0&amp;sitetype=fips&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=44.963469953193,-93.2677936369265", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">2743000</t>
@@ -1517,10 +1517,10 @@
     <t xml:space="preserve">Minnesota</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?fips=2743306&amp;buffer=0&amp;sitenumber=-1&amp;sitetype=fips&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=44.9355319808696,-93.7107081310233", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?fips=2743306&amp;buffer=0&amp;sitetype=fips&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=44.9355319808697,-93.7107081310232", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">2743306</t>
@@ -5957,7 +5957,7 @@
         <v>0.812974644245306</v>
       </c>
       <c r="S2" s="28" t="n">
-        <v>1.08127412769043</v>
+        <v>1.08127412769044</v>
       </c>
       <c r="T2" s="28" t="n">
         <v>0.601493907545558</v>
@@ -6041,7 +6041,7 @@
         <v>1.3170152917016</v>
       </c>
       <c r="AU2" s="28" t="n">
-        <v>1.41815394218697</v>
+        <v>1.41815394218698</v>
       </c>
       <c r="AV2" s="28" t="n">
         <v>2.20653957742285</v>
@@ -7141,7 +7141,7 @@
         <v>127.278893976343</v>
       </c>
       <c r="PE2" s="25" t="n">
-        <v>100.365437071176</v>
+        <v>100.365437071175</v>
       </c>
       <c r="PF2" s="25" t="n">
         <v>134.861992779648</v>
@@ -7165,7 +7165,7 @@
         <v>173.449621144755</v>
       </c>
       <c r="PM2" s="25" t="n">
-        <v>44.1921717053729</v>
+        <v>44.192171705373</v>
       </c>
       <c r="PN2" s="25" t="n">
         <v>165.50400143161</v>
@@ -7279,7 +7279,7 @@
         <v>148.045637607575</v>
       </c>
       <c r="QY2" s="23" t="n">
-        <v>57.3795365809011</v>
+        <v>57.3795365809129</v>
       </c>
     </row>
     <row r="3">
@@ -7416,7 +7416,7 @@
         <v>0.342210758140575</v>
       </c>
       <c r="AU3" s="28" t="n">
-        <v>0.537910179587159</v>
+        <v>0.537910179587158</v>
       </c>
       <c r="AV3" s="28" t="n">
         <v>0.160422268053344</v>
@@ -7437,7 +7437,7 @@
         <v>0.23144979948895</v>
       </c>
       <c r="BB3" s="28" t="n">
-        <v>0.0965414570879532</v>
+        <v>0.0965414570879531</v>
       </c>
       <c r="BC3" s="28" t="n">
         <v>0.0259959422919436</v>
@@ -7503,7 +7503,7 @@
         <v>0.313333788166709</v>
       </c>
       <c r="BX3" s="28" t="n">
-        <v>0.805854765268448</v>
+        <v>0.805854765268447</v>
       </c>
       <c r="BY3" s="30" t="n">
         <v>0.363895727164223</v>
@@ -8519,7 +8519,7 @@
         <v>7.07557891337977</v>
       </c>
       <c r="PF3" s="25" t="n">
-        <v>24.1479683249791</v>
+        <v>24.147968324979</v>
       </c>
       <c r="PG3" s="25" t="n">
         <v>9.42138859407052</v>
@@ -8654,7 +8654,7 @@
         <v>0</v>
       </c>
       <c r="QY3" s="23" t="n">
-        <v>30.9768218053203</v>
+        <v>30.9768218053251</v>
       </c>
     </row>
   </sheetData>
@@ -10523,7 +10523,7 @@
         <v>1.43296505903985</v>
       </c>
       <c r="BM2" s="28" t="n">
-        <v>2.11739173358115</v>
+        <v>2.11739173358114</v>
       </c>
       <c r="BN2" s="28" t="n">
         <v>1.26360477486346</v>
@@ -10664,7 +10664,7 @@
         <v>0.00748251633940476</v>
       </c>
       <c r="DH2" s="30" t="n">
-        <v>0.00309425256640238</v>
+        <v>0.00309425256640237</v>
       </c>
       <c r="DI2" s="30" t="n">
         <v>0.0108971534326254</v>
@@ -11542,7 +11542,7 @@
         <v>0.000372222120103671</v>
       </c>
       <c r="OV2" s="30" t="n">
-        <v>0.0439176148374171</v>
+        <v>0.043917614837417</v>
       </c>
       <c r="OW2" s="30" t="n">
         <v>0.0766915427458045</v>
@@ -11707,7 +11707,7 @@
         <v>146.30794436588</v>
       </c>
       <c r="QY2" s="23" t="n">
-        <v>88.3563583862214</v>
+        <v>88.356358386238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>